<commit_message>
Add QC pass + Employees/Influencers and Repeat Customers consolidation sheets
- QC verified: 190 complimentary deals since 1 Jan 2026, all Amount=0,
  clean date-cutoff boundary, 0 unparsed item lines; flagged 32 zero-value
  sample sends included in unit counts but not in AED value.
- New 'Employees & Influencers' sheet: named recipients matched by exact
  name (avoids Abboud vs Yana Abboud; consolidates Eugene Bolok's two IDs).
- New 'Repeat Customers' sheet: customers with 2+ complimentary checkouts,
  with food and value.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ad4mjJESUsMUoCNGegANgD
</commit_message>
<xml_diff>
--- a/Complimentary_Checkouts_Report_2026.xlsx
+++ b/Complimentary_Checkouts_Report_2026.xlsx
@@ -13,6 +13,8 @@
     <sheet name="Customers &amp; Products" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Products Given Away" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="100pct Discounted (appendix)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Employees &amp; Influencers" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Repeat Customers" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,8 +59,23 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E2E"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E2E"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -68,6 +85,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002E7D46"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6F0E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CDE3D3"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,6 +146,15 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -18211,4 +18247,1442 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Consolidated Complimentary Food — Named Recipients</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Complimentary checkouts since 1 January 2026, matched by exact customer name</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Comp Deals</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Product Value (AED)</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Delivery Waived</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Total Value (AED)</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>Products Received (qty x item)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>EMPLOYEES</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="n"/>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="16" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Eugene Bolok</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D6" s="12" t="n">
+        <v>3207.95</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>3607.95</v>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>16 x 1Kg Camel with Quinoa - Subsc.
+11 x 1Kg Camel with Dates - Subsc.
+11 x 1Kg Lamb with Apple - Subsc.
+6 x 1Kg Beef with Beetroot - Subsc.
+6 x 1Kg Turkey with Quinoa - Subsc
+4 x Berry Turkey 120g
+4 x 1Kg Turkey with Honey - Subsc.
+4 x 1Kg Grain Free Chicken - Subsc.
+2 x Camel Bone Broth 250g
+1 x Color My Plate 6 Pack
+1 x Gentle Turkey 120g
+1 x 1Kg Chicken with Banana - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Andrea Petrovic</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>1160.25</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="F7" s="12" t="n">
+        <v>1260.25</v>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>14 x 1Kg Beef with Beetroot - Subsc.
+10 x Beef Pâté Sample - 80g
+6 x 1Kg Camel with Dates - Subsc.
+4 x 1Kg Chicken with Banana - Subsc.
+2 x 1Kg Lamb with Apple - Subsc.
+1 x Samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Abboud</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>1670.13</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>225</v>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>1895.13</v>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>20 x Cat Food Sample
+15 x 80g Chicken with Mussels Pâté - Subsc.
+13 x 80g Duck with Tuna Pâté - Subsc.
+8 x Chicken Pâté 80g
+8 x Beef Pâté 80g
+7 x 1Kg Beef with Beetroot - Subsc.
+7 x 1Kg Turkey with Honey - Subsc.
+6 x 1Kg Camel with Dates - Subsc.
+6 x 1Kg Lamb with Apple - Subsc.
+5 x 80g Chicken Pâté - Subsc.
+5 x 80g Beef Pâté - Subsc.
+5 x Duck with Tuna Pâté Sample - 80g
+5 x Chicken Pâté Sample - 80g
+5 x Beef Pâté Sample - 80g
+2 x 1Kg Chicken with Banana - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>EMPLOYEES — Subtotal</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n"/>
+      <c r="C9" s="17" t="n">
+        <v>29</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>6038.33</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>725</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>6763.33</v>
+      </c>
+      <c r="G9" s="18" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>INFLUENCERS</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="16" t="n"/>
+      <c r="D11" s="16" t="n"/>
+      <c r="E11" s="16" t="n"/>
+      <c r="F11" s="16" t="n"/>
+      <c r="G11" s="16" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Fatima Tehrani</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="12" t="n">
+        <v>1502.64</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="F12" s="12" t="n">
+        <v>1552.64</v>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>36 x 1Kg Beef with Beetroot - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Tiakala Sangtam</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <v>2319.94</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>125</v>
+      </c>
+      <c r="F13" s="12" t="n">
+        <v>2444.94</v>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>38 x 1Kg Camel with Quinoa - Subsc.
+8 x 1Kg Chicken with Banana - Subsc.
+4 x 1Kg Wundercare Digestive Low Fat - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Clair De Valk</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="12" t="n">
+        <v>2055.24</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="F14" s="12" t="n">
+        <v>2255.24</v>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>24 x 1Kg Turkey with Honey - Subsc.
+10 x 1Kg Wundercare Digestive Moderate Fat - Subsc.
+6 x 1Kg Chicken with Banana - Subsc.
+1 x Color My Plate 6 Pack
+1 x Camel Bone Broth 250g</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Malak Alsaffar</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>524.09</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <v>624.09</v>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>4 x 1Kg Chicken with Banana - Subsc.
+4 x 1Kg Camel with Dates - Subsc.
+4 x 1Kg Turkey with Honey - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Stephy Augustine</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <v>303.04</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="F16" s="12" t="n">
+        <v>353.04</v>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>2 x 1Kg Beef with Beetroot - Subsc.
+2 x 1Kg Camel with Dates - Subsc.
+2 x 1Kg Turkey with Quinoa - Subsc</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>INFLUENCERS — Subtotal</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="D17" s="19" t="n">
+        <v>6704.95</v>
+      </c>
+      <c r="E17" s="19" t="n">
+        <v>525</v>
+      </c>
+      <c r="F17" s="19" t="n">
+        <v>7229.95</v>
+      </c>
+      <c r="G17" s="18" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL (named recipients)</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="D19" s="21" t="n">
+        <v>12743.28</v>
+      </c>
+      <c r="E19" s="21" t="n">
+        <v>1250</v>
+      </c>
+      <c r="F19" s="21" t="n">
+        <v>13993.28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Repeat Complimentary Customers (2+ free checkouts since 1 Jan 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Customer Name</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Customer #(s)</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Comp Deals</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Product Value (AED)</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Delivery Waived</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>Total Value (AED)</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>Products Received (qty x item)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Everything Dog Retail</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>40139</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>6810</v>
+      </c>
+      <c r="F4" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="G4" s="12" t="n">
+        <v>6835</v>
+      </c>
+      <c r="H4" s="11" t="inlineStr">
+        <is>
+          <t>46 x Beef with Beetroot 1kg
+26 x Lamb with Apple 1kg
+13 x Turkey with Honey 1kg
+13 x Turkey with Quinoa 1kg
+10 x Camel with Dates 1kg
+10 x Camel with Quinoa 1kg
+8 x Chicken with Banana 1kg
+8 x Grain-free Chicken 1kg
+4 x Camel Bone Broth 250g
+4 x Pumpkin Purée 500g
+3 x Gentle Turkey 120g
+3 x Berry Turkey 120g
+3 x Super Green Turkey 120g
+1 x Camel Bone Broth (3 Pieces)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Eugene Bolok</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>29894</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>3207.95</v>
+      </c>
+      <c r="F5" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>3607.95</v>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>16 x 1Kg Camel with Quinoa - Subsc.
+11 x 1Kg Camel with Dates - Subsc.
+11 x 1Kg Lamb with Apple - Subsc.
+6 x 1Kg Beef with Beetroot - Subsc.
+6 x 1Kg Turkey with Quinoa - Subsc
+4 x Berry Turkey 120g
+4 x 1Kg Turkey with Honey - Subsc.
+4 x 1Kg Grain Free Chicken - Subsc.
+2 x Camel Bone Broth 250g
+1 x Color My Plate 6 Pack
+1 x Gentle Turkey 120g
+1 x 1Kg Chicken with Banana - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Tiakala Sangtam</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>24021</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>2319.94</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>125</v>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>2444.94</v>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>38 x 1Kg Camel with Quinoa - Subsc.
+8 x 1Kg Chicken with Banana - Subsc.
+4 x 1Kg Wundercare Digestive Low Fat - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Clair De Valk</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>26282</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>2055.24</v>
+      </c>
+      <c r="F7" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>2255.24</v>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>24 x 1Kg Turkey with Honey - Subsc.
+10 x 1Kg Wundercare Digestive Moderate Fat - Subsc.
+6 x 1Kg Chicken with Banana - Subsc.
+1 x Color My Plate 6 Pack
+1 x Camel Bone Broth 250g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Sarah Caroline Tamsin Ramsey</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>23877</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>1875.77</v>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="G8" s="12" t="n">
+        <v>2025.77</v>
+      </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>15 x 80g Duck with Tuna Pâté - Subsc.
+13 x 1Kg Beef with Beetroot - Subsc.
+10 x 1Kg Camel with Dates - Subsc.
+10 x 80g Beef with Sardines Pâté - Subsc.
+9 x 1Kg Lamb with Apple - Subsc.
+5 x 80g Chicken with Mussels Pâté - Subsc.
+2 x 1Kg Wundercare Digestive Moderate Fat - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Abboud</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>888</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>1670.13</v>
+      </c>
+      <c r="F9" s="12" t="n">
+        <v>225</v>
+      </c>
+      <c r="G9" s="12" t="n">
+        <v>1895.13</v>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>20 x Cat Food Sample
+15 x 80g Chicken with Mussels Pâté - Subsc.
+13 x 80g Duck with Tuna Pâté - Subsc.
+8 x Chicken Pâté 80g
+8 x Beef Pâté 80g
+7 x 1Kg Beef with Beetroot - Subsc.
+7 x 1Kg Turkey with Honey - Subsc.
+6 x 1Kg Camel with Dates - Subsc.
+6 x 1Kg Lamb with Apple - Subsc.
+5 x 80g Chicken Pâté - Subsc.
+5 x 80g Beef Pâté - Subsc.
+5 x Duck with Tuna Pâté Sample - 80g
+5 x Chicken Pâté Sample - 80g
+5 x Beef Pâté Sample - 80g
+2 x 1Kg Chicken with Banana - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Vishaal S Shah</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>22652</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>1551.85</v>
+      </c>
+      <c r="F10" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="G10" s="12" t="n">
+        <v>1601.85</v>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>17 x 1Kg Wundercare Liver Copper-Restricted - Subsc.
+4 x 1Kg Beef with Beetroot - Subsc.
+3 x 1Kg Lamb with Apple - Subsc.
+2 x 1Kg Grain Free Chicken - Subsc.
+2 x 1Kg Camel with Dates - Subsc.
+2 x 1Kg Turkey with Honey - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Fatima Tehrani</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>26492</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>1502.64</v>
+      </c>
+      <c r="F11" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="G11" s="12" t="n">
+        <v>1552.64</v>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>36 x 1Kg Beef with Beetroot - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Andrea Petrovic</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>1315</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>1160.25</v>
+      </c>
+      <c r="F12" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="G12" s="12" t="n">
+        <v>1260.25</v>
+      </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>14 x 1Kg Beef with Beetroot - Subsc.
+10 x Beef Pâté Sample - 80g
+6 x 1Kg Camel with Dates - Subsc.
+4 x 1Kg Chicken with Banana - Subsc.
+2 x 1Kg Lamb with Apple - Subsc.
+1 x Samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Rajiv Prasad</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>29699</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>886.54</v>
+      </c>
+      <c r="F13" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="G13" s="12" t="n">
+        <v>936.54</v>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t>6 x 1Kg Lamb with Apple - Subsc.
+6 x 1Kg Turkey with Honey - Subsc.
+3 x 1Kg Camel with Dates - Subsc.
+2 x 1Kg Chicken with Banana - Subsc.
+1 x 1Kg Beef with Beetroot - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Kelly Johnston</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>27647</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>771.41</v>
+      </c>
+      <c r="F14" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="G14" s="12" t="n">
+        <v>846.41</v>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>7 x 1Kg Camel with Dates - Subsc.
+6 x 1Kg Lamb with Apple - Subsc.
+1 x Camel with Dates 1kg
+1 x Camel with Quinoa 1kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Panacea Vets</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>42280</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>657.6</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="G15" s="12" t="n">
+        <v>682.6</v>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>30 x Duck with Tuna Pâté 80g
+30 x Chicken Pâté 80g
+10 x Gentle Turkey 120g
+10 x Beef with Sardines Pâté
+5 x Beef Pâté 80g
+3 x Camel Bone Broth 250g</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Kate George</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>27186</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>604.99</v>
+      </c>
+      <c r="F16" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="G16" s="12" t="n">
+        <v>654.99</v>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t>4 x 1Kg Lamb with Apple - Subsc.
+4 x 1Kg Camel with Dates - Subsc.
+4 x 1Kg Turkey with Honey - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Cong Luo</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>27339</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="12" t="n">
+        <v>474.81</v>
+      </c>
+      <c r="F17" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="G17" s="12" t="n">
+        <v>524.8099999999999</v>
+      </c>
+      <c r="H17" s="11" t="inlineStr">
+        <is>
+          <t>9 x 1Kg Camel with Quinoa - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Akshay Sonawane</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>23819</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>433.99</v>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="G18" s="12" t="n">
+        <v>483.99</v>
+      </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t>16 x Cat Food Sample
+5 x 1Kg Chicken with Banana - Subsc.
+2 x 1Kg Grain Free Chicken - Subsc.
+1 x 1Kg Beef with Beetroot - Subsc.
+1 x 1Kg Lamb with Apple - Subsc.
+1 x 1Kg Camel with Dates - Subsc.
+1 x 1Kg Turkey with Quinoa - Subsc</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Nicola Schmitz</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>26097</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <v>389.84</v>
+      </c>
+      <c r="F19" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="G19" s="12" t="n">
+        <v>439.84</v>
+      </c>
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t>4 x 1Kg Camel with Dates - Subsc.
+2 x 1Kg Grain Free Chicken - Subsc.
+2 x 1Kg Turkey with Quinoa - Subsc</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Taskeen Moolla</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>26891</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="12" t="n">
+        <v>389.2</v>
+      </c>
+      <c r="F20" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="G20" s="12" t="n">
+        <v>414.2</v>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>35 x 80g Duck with Tuna Pâté - Subsc.
+23 x Beef Pâté 80g</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Zak</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>41550</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="12" t="n">
+        <v>364</v>
+      </c>
+      <c r="F21" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="G21" s="12" t="n">
+        <v>414</v>
+      </c>
+      <c r="H21" s="11" t="inlineStr">
+        <is>
+          <t>4 x Chicken with Banana 1kg
+4 x Turkey with Honey 1kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Diana Stepan</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>27253</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="12" t="n">
+        <v>275.48</v>
+      </c>
+      <c r="F22" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="G22" s="12" t="n">
+        <v>350.48</v>
+      </c>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>3 x 1Kg Camel with Quinoa - Subsc.
+2 x Camel with Quinoa 1kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Mariam</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>29648, 40932</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="12" t="n">
+        <v>169.6</v>
+      </c>
+      <c r="F23" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="G23" s="12" t="n">
+        <v>219.6</v>
+      </c>
+      <c r="H23" s="11" t="inlineStr">
+        <is>
+          <t>2 x 1Kg Chicken with Banana - Subsc.
+2 x 1Kg Turkey with Honey - Subsc.
+1 x Samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Erika Belaja</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>40937</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="12" t="n">
+        <v>133.6</v>
+      </c>
+      <c r="F24" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="G24" s="12" t="n">
+        <v>183.6</v>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>1 x 1Kg Chicken with Banana - Subsc.
+1 x 1Kg Camel with Dates - Subsc.
+1 x 1Kg Beef with Beetroot - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Second Chance Animal Sanctuary</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>29813</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E25" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="12" t="n">
+        <v>175</v>
+      </c>
+      <c r="G25" s="12" t="n">
+        <v>175</v>
+      </c>
+      <c r="H25" s="11" t="inlineStr">
+        <is>
+          <t>10 x Samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Alessandra Fuscaldo</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>42050</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="12" t="n">
+        <v>106.12</v>
+      </c>
+      <c r="F26" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="G26" s="12" t="n">
+        <v>131.12</v>
+      </c>
+      <c r="H26" s="11" t="inlineStr">
+        <is>
+          <t>12 x 80g Duck with Tuna Pâté - Subsc.
+4 x 80g Chicken Pâté - Subsc.
+4 x 80g Beef Pâté - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Dr. Susan Aylott</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>40709</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="G27" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="H27" s="11" t="inlineStr">
+        <is>
+          <t>5 x 80g Duck with Tuna Pâté - Subsc.
+5 x 80g Chicken Pâté - Subsc.
+5 x 80g Beef Pâté - Subsc.
+1 x Samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL (repeat customers)</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="n"/>
+      <c r="C28" s="18" t="n"/>
+      <c r="D28" s="17" t="n">
+        <v>98</v>
+      </c>
+      <c r="E28" s="19" t="n">
+        <v>27810.95</v>
+      </c>
+      <c r="F28" s="19" t="n">
+        <v>2150</v>
+      </c>
+      <c r="G28" s="19" t="n">
+        <v>29960.95</v>
+      </c>
+      <c r="H28" s="18" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix: count all free deals (complimentary + 100%-discounted) for named recipients
Mariam Lando and other influencers receive free product mainly via
100%-discounted subscriptions, not the Complimentary payment type. The
Employees & Influencers and Repeat Customers sheets now aggregate over the
full free universe (Amount invoiced = 0 = complimentary + 100%-discounted),
with Comp / 100%-Disc split columns for transparency.

- Influencers: 10 -> 30 free deals; gross AED 6.7k -> 21.8k.
- Mariam Lando now correctly shows 4 free deals (was 1 zero-value sample).
- Summary block D and Repeat Customers updated to match (repeat 23 -> 26).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ad4mjJESUsMUoCNGegANgD
</commit_message>
<xml_diff>
--- a/Complimentary_Checkouts_Report_2026.xlsx
+++ b/Complimentary_Checkouts_Report_2026.xlsx
@@ -517,14 +517,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -685,7 +687,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>C. COMBINED TOTAL GIVEN AWAY FREE</t>
+          <t>C. COMBINED TOTAL GIVEN AWAY FREE (A + B)</t>
         </is>
       </c>
     </row>
@@ -712,7 +714,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>D. EMPLOYEE &amp; INFLUENCER COMPLIMENTARY (named recipients)</t>
+          <t>D. EMPLOYEE &amp; INFLUENCER FREE PRODUCT (complimentary + 100%-discounted)</t>
         </is>
       </c>
     </row>
@@ -724,20 +726,30 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Deals</t>
+          <t>Free Deals</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
+          <t>of which Comp</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>of which 100%-Disc</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
           <t>Product Value</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="F26" s="8" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="G26" s="8" t="inlineStr">
         <is>
           <t>Total Value</t>
         </is>
@@ -752,13 +764,19 @@
       <c r="B27" t="n">
         <v>29</v>
       </c>
-      <c r="C27" s="7" t="n">
+      <c r="C27" t="n">
+        <v>29</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="7" t="n">
         <v>6038.33</v>
       </c>
-      <c r="D27" s="7" t="n">
+      <c r="F27" s="7" t="n">
         <v>725</v>
       </c>
-      <c r="E27" s="7" t="n">
+      <c r="G27" s="7" t="n">
         <v>6763.33</v>
       </c>
     </row>
@@ -769,16 +787,22 @@
         </is>
       </c>
       <c r="B28" t="n">
+        <v>30</v>
+      </c>
+      <c r="C28" t="n">
         <v>10</v>
       </c>
-      <c r="C28" s="7" t="n">
-        <v>6704.95</v>
-      </c>
-      <c r="D28" s="7" t="n">
+      <c r="D28" t="n">
+        <v>20</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>21782.82</v>
+      </c>
+      <c r="F28" s="7" t="n">
         <v>550</v>
       </c>
-      <c r="E28" s="7" t="n">
-        <v>7254.95</v>
+      <c r="G28" s="7" t="n">
+        <v>22332.82</v>
       </c>
     </row>
     <row r="29">
@@ -788,16 +812,22 @@
         </is>
       </c>
       <c r="B29" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="C29" s="9" t="n">
         <v>39</v>
       </c>
-      <c r="C29" s="10" t="n">
-        <v>12743.28</v>
-      </c>
-      <c r="D29" s="10" t="n">
+      <c r="D29" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="E29" s="10" t="n">
+        <v>27821.15</v>
+      </c>
+      <c r="F29" s="10" t="n">
         <v>1275</v>
       </c>
-      <c r="E29" s="10" t="n">
-        <v>14018.28</v>
+      <c r="G29" s="10" t="n">
+        <v>29096.15</v>
       </c>
     </row>
     <row r="31">
@@ -13440,29 +13470,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Consolidated Complimentary Food — Named Recipients</t>
+          <t>Consolidated Free Product — Named Recipients</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Complimentary checkouts since 1 Jan 2026. Names matched exactly; Mariam Lando matched by Customer #40932.</t>
+          <t>ALL free deals since 1 Jan 2026 = Complimentary + 100%-discounted (zero invoiced). Mariam Lando matched by Customer #40932.</t>
         </is>
       </c>
     </row>
@@ -13479,25 +13511,35 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Comp Deals</t>
+          <t>Free Deals</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
+          <t>Comp</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>100%-Disc</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
           <t>Gross Value (AED)</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>Delivery Waived</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>Total Value (AED)</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>Products Received (qty x item)</t>
         </is>
@@ -13515,6 +13557,8 @@
       <c r="E5" s="18" t="n"/>
       <c r="F5" s="18" t="n"/>
       <c r="G5" s="18" t="n"/>
+      <c r="H5" s="18" t="n"/>
+      <c r="I5" s="18" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -13530,16 +13574,22 @@
       <c r="C6" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="14" t="n">
         <v>3207.95</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="G6" s="14" t="n">
         <v>400</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="H6" s="7" t="n">
         <v>3607.95</v>
       </c>
-      <c r="G6" s="12" t="inlineStr">
+      <c r="I6" s="12" t="inlineStr">
         <is>
           <t>16 x 1Kg Camel with Quinoa - Subsc.
 11 x 1Kg Camel with Dates - Subsc.
@@ -13570,16 +13620,22 @@
       <c r="C7" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="14" t="n">
         <v>1160.25</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="G7" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="H7" s="7" t="n">
         <v>1260.25</v>
       </c>
-      <c r="G7" s="12" t="inlineStr">
+      <c r="I7" s="12" t="inlineStr">
         <is>
           <t>14 x 1Kg Beef with Beetroot - Subsc.
 10 x Beef Pâté Sample - 80g
@@ -13604,16 +13660,22 @@
       <c r="C8" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="14" t="n">
         <v>1670.13</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="G8" s="14" t="n">
         <v>225</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="H8" s="7" t="n">
         <v>1895.13</v>
       </c>
-      <c r="G8" s="12" t="inlineStr">
+      <c r="I8" s="12" t="inlineStr">
         <is>
           <t>20 x Cat Food Sample
 15 x 80g Chicken with Mussels Pâté - Subsc.
@@ -13643,16 +13705,22 @@
       <c r="C9" s="9" t="n">
         <v>29</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="10" t="n">
         <v>6038.33</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="G9" s="10" t="n">
         <v>725</v>
       </c>
-      <c r="F9" s="10" t="n">
+      <c r="H9" s="10" t="n">
         <v>6763.33</v>
       </c>
-      <c r="G9" s="13" t="n"/>
+      <c r="I9" s="13" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
@@ -13666,6 +13734,8 @@
       <c r="E11" s="18" t="n"/>
       <c r="F11" s="18" t="n"/>
       <c r="G11" s="18" t="n"/>
+      <c r="H11" s="18" t="n"/>
+      <c r="I11" s="18" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
@@ -13681,16 +13751,22 @@
       <c r="C12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="14" t="n">
         <v>1502.64</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="G12" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="F12" s="14" t="n">
+      <c r="H12" s="7" t="n">
         <v>1552.64</v>
       </c>
-      <c r="G12" s="12" t="inlineStr">
+      <c r="I12" s="12" t="inlineStr">
         <is>
           <t>36 x 1Kg Beef with Beetroot - Subsc.</t>
         </is>
@@ -13708,22 +13784,33 @@
         </is>
       </c>
       <c r="C13" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D13" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="D13" s="14" t="n">
-        <v>2319.94</v>
-      </c>
-      <c r="E13" s="14" t="n">
+      <c r="E13" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="14" t="n">
+        <v>8244.959999999999</v>
+      </c>
+      <c r="G13" s="14" t="n">
         <v>125</v>
       </c>
-      <c r="F13" s="14" t="n">
-        <v>2444.94</v>
-      </c>
-      <c r="G13" s="12" t="inlineStr">
-        <is>
-          <t>38 x 1Kg Camel with Quinoa - Subsc.
-8 x 1Kg Chicken with Banana - Subsc.
-4 x 1Kg Wundercare Digestive Low Fat - Subsc.</t>
+      <c r="H13" s="7" t="n">
+        <v>8369.959999999999</v>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>118 x 1Kg Camel with Quinoa - Subsc.
+35 x 1Kg Wundercare Digestive Low Fat - Subsc.
+35 x 80g Duck with Tuna Pâté - Subsc.
+31 x Cat Food Sample
+27 x 1Kg Chicken with Banana - Subsc.
+2 x Chicken Pâté Sample - 80g
+2 x Beef Pâté Sample - 80g
+1 x 1Kg Beef with Beetroot - Subsc.</t>
         </is>
       </c>
     </row>
@@ -13739,23 +13826,29 @@
         </is>
       </c>
       <c r="C14" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D14" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="14" t="n">
-        <v>2055.24</v>
-      </c>
-      <c r="E14" s="14" t="n">
+      <c r="E14" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>7189.85</v>
+      </c>
+      <c r="G14" s="14" t="n">
         <v>200</v>
       </c>
-      <c r="F14" s="14" t="n">
-        <v>2255.24</v>
-      </c>
-      <c r="G14" s="12" t="inlineStr">
-        <is>
-          <t>24 x 1Kg Turkey with Honey - Subsc.
+      <c r="H14" s="7" t="n">
+        <v>7389.85</v>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>171 x 1Kg Chicken with Banana - Subsc.
+24 x 1Kg Turkey with Honey - Subsc.
 10 x 1Kg Wundercare Digestive Moderate Fat - Subsc.
-6 x 1Kg Chicken with Banana - Subsc.
-1 x Color My Plate 6 Pack
+2 x Color My Plate 6 Pack
 1 x Camel Bone Broth 250g</t>
         </is>
       </c>
@@ -13772,22 +13865,28 @@
         </is>
       </c>
       <c r="C15" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="14" t="n">
-        <v>524.09</v>
-      </c>
-      <c r="E15" s="14" t="n">
+      <c r="E15" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="F15" s="14" t="n">
+        <v>3740.47</v>
+      </c>
+      <c r="G15" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="F15" s="14" t="n">
-        <v>624.09</v>
-      </c>
-      <c r="G15" s="12" t="inlineStr">
-        <is>
-          <t>4 x 1Kg Chicken with Banana - Subsc.
-4 x 1Kg Camel with Dates - Subsc.
-4 x 1Kg Turkey with Honey - Subsc.</t>
+      <c r="H15" s="7" t="n">
+        <v>3840.47</v>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>28 x 1Kg Chicken with Banana - Subsc.
+28 x 1Kg Camel with Dates - Subsc.
+28 x 1Kg Turkey with Honey - Subsc.</t>
         </is>
       </c>
     </row>
@@ -13805,16 +13904,22 @@
       <c r="C16" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="14" t="n">
+      <c r="D16" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="14" t="n">
         <v>303.04</v>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="G16" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="F16" s="14" t="n">
+      <c r="H16" s="7" t="n">
         <v>353.04</v>
       </c>
-      <c r="G16" s="12" t="inlineStr">
+      <c r="I16" s="12" t="inlineStr">
         <is>
           <t>2 x 1Kg Beef with Beetroot - Subsc.
 2 x 1Kg Camel with Dates - Subsc.
@@ -13834,20 +13939,29 @@
         </is>
       </c>
       <c r="C17" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="14" t="n">
-        <v>25</v>
+      <c r="E17" s="11" t="n">
+        <v>3</v>
       </c>
       <c r="F17" s="14" t="n">
-        <v>25</v>
-      </c>
-      <c r="G17" s="12" t="inlineStr">
-        <is>
-          <t>1 x Samples</t>
+        <v>801.86</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>826.86</v>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>10 x 1Kg Camel with Dates - Subsc.
+3 x Color My Plate 6 Pack
+2 x 1Kg Chicken with Banana - Subsc.
+1 x Samples</t>
         </is>
       </c>
     </row>
@@ -13859,18 +13973,24 @@
       </c>
       <c r="B18" s="13" t="n"/>
       <c r="C18" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="D18" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="D18" s="10" t="n">
-        <v>6704.95</v>
-      </c>
-      <c r="E18" s="10" t="n">
+      <c r="E18" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>21782.82</v>
+      </c>
+      <c r="G18" s="10" t="n">
         <v>550</v>
       </c>
-      <c r="F18" s="10" t="n">
-        <v>7254.95</v>
-      </c>
-      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="10" t="n">
+        <v>22332.82</v>
+      </c>
+      <c r="I18" s="13" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="19" t="inlineStr">
@@ -13880,18 +14000,20 @@
       </c>
       <c r="B20" s="13" t="n"/>
       <c r="C20" s="9" t="n">
-        <v>39</v>
-      </c>
-      <c r="D20" s="10" t="n">
-        <v>12743.28</v>
-      </c>
-      <c r="E20" s="10" t="n">
+        <v>59</v>
+      </c>
+      <c r="D20" s="13" t="n"/>
+      <c r="E20" s="13" t="n"/>
+      <c r="F20" s="10" t="n">
+        <v>27821.15</v>
+      </c>
+      <c r="G20" s="10" t="n">
         <v>1275</v>
       </c>
-      <c r="F20" s="10" t="n">
-        <v>14018.28</v>
-      </c>
-      <c r="G20" s="13" t="n"/>
+      <c r="H20" s="10" t="n">
+        <v>29096.15</v>
+      </c>
+      <c r="I20" s="13" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13904,30 +14026,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Repeat Complimentary Customers (2+ free checkouts since 1 Jan 2026)</t>
+          <t>Repeat Free Customers (2+ free checkouts since 1 Jan 2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Grouped by Customer # (distinct accounts with the same name kept separate)</t>
+          <t>Free = complimentary + 100%-discounted. Grouped by Customer # (distinct accounts kept separate).</t>
         </is>
       </c>
     </row>
@@ -13949,25 +14073,35 @@
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Comp Deals</t>
+          <t>Free Deals</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
+          <t>Comp</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>100%-Disc</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
           <t>Gross Value (AED)</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>Delivery Waived</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Total Value (AED)</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Products Received (qty x item)</t>
         </is>
@@ -13975,31 +14109,124 @@
     </row>
     <row r="4">
       <c r="A4" s="11" t="n">
+        <v>24021</v>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Tiakala Sangtam</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>8244.959999999999</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <v>125</v>
+      </c>
+      <c r="I4" s="14" t="n">
+        <v>8369.959999999999</v>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>118 x 1Kg Camel with Quinoa - Subsc.
+35 x 1Kg Wundercare Digestive Low Fat - Subsc.
+35 x 80g Duck with Tuna Pâté - Subsc.
+31 x Cat Food Sample
+27 x 1Kg Chicken with Banana - Subsc.
+2 x Chicken Pâté Sample - 80g
+2 x Beef Pâté Sample - 80g
+1 x 1Kg Beef with Beetroot - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="n">
+        <v>26282</v>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Clair De Valk</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>7189.85</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>7389.85</v>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>171 x 1Kg Chicken with Banana - Subsc.
+24 x 1Kg Turkey with Honey - Subsc.
+10 x 1Kg Wundercare Digestive Moderate Fat - Subsc.
+2 x Color My Plate 6 Pack
+1 x Camel Bone Broth 250g</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="n">
         <v>40139</v>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Everything Dog Retail</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D4" s="11" t="n">
+      <c r="D6" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="E4" s="14" t="n">
+      <c r="E6" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="14" t="n">
         <v>6810</v>
       </c>
-      <c r="F4" s="14" t="n">
-        <v>25</v>
-      </c>
-      <c r="G4" s="14" t="n">
+      <c r="H6" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="I6" s="14" t="n">
         <v>6835</v>
       </c>
-      <c r="H4" s="12" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>46 x Beef with Beetroot 1kg
 26 x Lamb with Apple 1kg
@@ -14018,33 +14245,79 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="11" t="n">
+    <row r="7">
+      <c r="A7" s="11" t="n">
+        <v>40422</v>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Malak Alsaffar</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>3740.47</v>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>3840.47</v>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>28 x 1Kg Chicken with Banana - Subsc.
+28 x 1Kg Camel with Dates - Subsc.
+28 x 1Kg Turkey with Honey - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="n">
         <v>29894</v>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Eugene Bolok</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D8" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="E5" s="14" t="n">
+      <c r="E8" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="14" t="n">
         <v>3207.95</v>
       </c>
-      <c r="F5" s="14" t="n">
+      <c r="H8" s="14" t="n">
         <v>400</v>
       </c>
-      <c r="G5" s="14" t="n">
+      <c r="I8" s="14" t="n">
         <v>3607.95</v>
       </c>
-      <c r="H5" s="12" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>16 x 1Kg Camel with Quinoa - Subsc.
 11 x 1Kg Camel with Dates - Subsc.
@@ -14061,103 +14334,82 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="11" t="n">
-        <v>24021</v>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Tiakala Sangtam</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>Influencer</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="n">
+    <row r="9">
+      <c r="A9" s="11" t="n">
+        <v>22652</v>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Vishaal S Shah</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="14" t="n">
-        <v>2319.94</v>
-      </c>
-      <c r="F6" s="14" t="n">
-        <v>125</v>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>2444.94</v>
-      </c>
-      <c r="H6" s="12" t="inlineStr">
-        <is>
-          <t>38 x 1Kg Camel with Quinoa - Subsc.
-8 x 1Kg Chicken with Banana - Subsc.
-4 x 1Kg Wundercare Digestive Low Fat - Subsc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="n">
-        <v>26282</v>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>Clair De Valk</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>Influencer</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>2055.24</v>
-      </c>
-      <c r="F7" s="14" t="n">
-        <v>200</v>
-      </c>
-      <c r="G7" s="14" t="n">
-        <v>2255.24</v>
-      </c>
-      <c r="H7" s="12" t="inlineStr">
-        <is>
-          <t>24 x 1Kg Turkey with Honey - Subsc.
-10 x 1Kg Wundercare Digestive Moderate Fat - Subsc.
-6 x 1Kg Chicken with Banana - Subsc.
-1 x Color My Plate 6 Pack
-1 x Camel Bone Broth 250g</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="n">
+      <c r="F9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>2246.18</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>2296.18</v>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>25 x 1Kg Wundercare Liver Copper-Restricted - Subsc.
+10 x 1Kg Beef with Beetroot - Subsc.
+3 x 1Kg Lamb with Apple - Subsc.
+2 x 1Kg Grain Free Chicken - Subsc.
+2 x 1Kg Camel with Dates - Subsc.
+2 x 1Kg Turkey with Honey - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="n">
         <v>23877</v>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Sarah Caroline Tamsin Ramsey</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D10" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E10" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="14" t="n">
         <v>1875.77</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="H10" s="14" t="n">
         <v>150</v>
       </c>
-      <c r="G8" s="14" t="n">
+      <c r="I10" s="14" t="n">
         <v>2025.77</v>
       </c>
-      <c r="H8" s="12" t="inlineStr">
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>15 x 80g Duck with Tuna Pâté - Subsc.
 13 x 1Kg Beef with Beetroot - Subsc.
@@ -14169,33 +14421,39 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="11" t="n">
+    <row r="11">
+      <c r="A11" s="11" t="n">
         <v>888</v>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Abboud</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D11" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E11" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="14" t="n">
         <v>1670.13</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="H11" s="14" t="n">
         <v>225</v>
       </c>
-      <c r="G9" s="14" t="n">
+      <c r="I11" s="14" t="n">
         <v>1895.13</v>
       </c>
-      <c r="H9" s="12" t="inlineStr">
+      <c r="J11" s="12" t="inlineStr">
         <is>
           <t>20 x Cat Food Sample
 15 x 80g Chicken with Mussels Pâté - Subsc.
@@ -14215,102 +14473,116 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="11" t="n">
-        <v>22652</v>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>Vishaal S Shah</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>Customer</t>
-        </is>
-      </c>
-      <c r="D10" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>1551.85</v>
-      </c>
-      <c r="F10" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="G10" s="14" t="n">
-        <v>1601.85</v>
-      </c>
-      <c r="H10" s="12" t="inlineStr">
-        <is>
-          <t>17 x 1Kg Wundercare Liver Copper-Restricted - Subsc.
-4 x 1Kg Beef with Beetroot - Subsc.
-3 x 1Kg Lamb with Apple - Subsc.
-2 x 1Kg Grain Free Chicken - Subsc.
-2 x 1Kg Camel with Dates - Subsc.
-2 x 1Kg Turkey with Honey - Subsc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="11" t="n">
-        <v>26492</v>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>Fatima Tehrani</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>Influencer</t>
-        </is>
-      </c>
-      <c r="D11" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>1502.64</v>
-      </c>
-      <c r="F11" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="G11" s="14" t="n">
-        <v>1552.64</v>
-      </c>
-      <c r="H11" s="12" t="inlineStr">
-        <is>
-          <t>36 x 1Kg Beef with Beetroot - Subsc.</t>
-        </is>
-      </c>
-    </row>
     <row r="12">
       <c r="A12" s="11" t="n">
+        <v>40268</v>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Saneesha Pradeep</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>1755.74</v>
+      </c>
+      <c r="H12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="14" t="n">
+        <v>1755.74</v>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>24 x 1Kg Beef with Beetroot - Subsc.
+12 x 1Kg Turkey with Honey - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="n">
+        <v>26492</v>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Fatima Tehrani</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="14" t="n">
+        <v>1502.64</v>
+      </c>
+      <c r="H13" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="I13" s="14" t="n">
+        <v>1552.64</v>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>36 x 1Kg Beef with Beetroot - Subsc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="n">
         <v>1315</v>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Andrea Petrovic</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D14" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E14" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="14" t="n">
         <v>1160.25</v>
       </c>
-      <c r="F12" s="14" t="n">
+      <c r="H14" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="G12" s="14" t="n">
+      <c r="I14" s="14" t="n">
         <v>1260.25</v>
       </c>
-      <c r="H12" s="12" t="inlineStr">
+      <c r="J14" s="12" t="inlineStr">
         <is>
           <t>14 x 1Kg Beef with Beetroot - Subsc.
 10 x Beef Pâté Sample - 80g
@@ -14321,33 +14593,39 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="11" t="n">
+    <row r="15">
+      <c r="A15" s="11" t="n">
         <v>29699</v>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Rajiv Prasad</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D15" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="E15" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="14" t="n">
         <v>886.54</v>
       </c>
-      <c r="F13" s="14" t="n">
+      <c r="H15" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="G13" s="14" t="n">
+      <c r="I15" s="14" t="n">
         <v>936.54</v>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="J15" s="12" t="inlineStr">
         <is>
           <t>6 x 1Kg Lamb with Apple - Subsc.
 6 x 1Kg Turkey with Honey - Subsc.
@@ -14357,33 +14635,39 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="11" t="n">
+    <row r="16">
+      <c r="A16" s="11" t="n">
         <v>27647</v>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Kelly Johnston</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D16" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="E16" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="14" t="n">
         <v>771.41</v>
       </c>
-      <c r="F14" s="14" t="n">
+      <c r="H16" s="14" t="n">
         <v>75</v>
       </c>
-      <c r="G14" s="14" t="n">
+      <c r="I16" s="14" t="n">
         <v>846.41</v>
       </c>
-      <c r="H14" s="12" t="inlineStr">
+      <c r="J16" s="12" t="inlineStr">
         <is>
           <t>7 x 1Kg Camel with Dates - Subsc.
 6 x 1Kg Lamb with Apple - Subsc.
@@ -14392,33 +14676,80 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="11" t="n">
+    <row r="17">
+      <c r="A17" s="11" t="n">
+        <v>40932</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Mariam Lando</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>801.86</v>
+      </c>
+      <c r="H17" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="I17" s="14" t="n">
+        <v>826.86</v>
+      </c>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>10 x 1Kg Camel with Dates - Subsc.
+3 x Color My Plate 6 Pack
+2 x 1Kg Chicken with Banana - Subsc.
+1 x Samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="n">
         <v>42280</v>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Panacea Vets</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D18" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E18" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="14" t="n">
         <v>657.6</v>
       </c>
-      <c r="F15" s="14" t="n">
-        <v>25</v>
-      </c>
-      <c r="G15" s="14" t="n">
+      <c r="H18" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="I18" s="14" t="n">
         <v>682.6</v>
       </c>
-      <c r="H15" s="12" t="inlineStr">
+      <c r="J18" s="12" t="inlineStr">
         <is>
           <t>30 x Duck with Tuna Pâté 80g
 30 x Chicken Pâté 80g
@@ -14429,33 +14760,39 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="11" t="n">
+    <row r="19">
+      <c r="A19" s="11" t="n">
         <v>27186</v>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Kate George</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D16" s="11" t="n">
+      <c r="D19" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E19" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="14" t="n">
         <v>604.99</v>
       </c>
-      <c r="F16" s="14" t="n">
+      <c r="H19" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="G16" s="14" t="n">
+      <c r="I19" s="14" t="n">
         <v>654.99</v>
       </c>
-      <c r="H16" s="12" t="inlineStr">
+      <c r="J19" s="12" t="inlineStr">
         <is>
           <t>4 x 1Kg Lamb with Apple - Subsc.
 4 x 1Kg Camel with Dates - Subsc.
@@ -14463,65 +14800,77 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="11" t="n">
+    <row r="20">
+      <c r="A20" s="11" t="n">
         <v>27339</v>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>Cong Luo</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D17" s="11" t="n">
+      <c r="D20" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="14" t="n">
+      <c r="E20" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="14" t="n">
         <v>474.81</v>
       </c>
-      <c r="F17" s="14" t="n">
+      <c r="H20" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="G17" s="14" t="n">
+      <c r="I20" s="14" t="n">
         <v>524.8099999999999</v>
       </c>
-      <c r="H17" s="12" t="inlineStr">
+      <c r="J20" s="12" t="inlineStr">
         <is>
           <t>9 x 1Kg Camel with Quinoa - Subsc.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="11" t="n">
+    <row r="21">
+      <c r="A21" s="11" t="n">
         <v>23819</v>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Akshay Sonawane</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D18" s="11" t="n">
+      <c r="D21" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E18" s="14" t="n">
+      <c r="E21" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="14" t="n">
         <v>433.99</v>
       </c>
-      <c r="F18" s="14" t="n">
+      <c r="H21" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="G18" s="14" t="n">
+      <c r="I21" s="14" t="n">
         <v>483.99</v>
       </c>
-      <c r="H18" s="12" t="inlineStr">
+      <c r="J21" s="12" t="inlineStr">
         <is>
           <t>16 x Cat Food Sample
 5 x 1Kg Chicken with Banana - Subsc.
@@ -14533,33 +14882,39 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="11" t="n">
+    <row r="22">
+      <c r="A22" s="11" t="n">
         <v>26097</v>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Nicola Schmitz</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D19" s="11" t="n">
+      <c r="D22" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E19" s="14" t="n">
+      <c r="E22" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="14" t="n">
         <v>389.84</v>
       </c>
-      <c r="F19" s="14" t="n">
+      <c r="H22" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="G19" s="14" t="n">
+      <c r="I22" s="14" t="n">
         <v>439.84</v>
       </c>
-      <c r="H19" s="12" t="inlineStr">
+      <c r="J22" s="12" t="inlineStr">
         <is>
           <t>4 x 1Kg Camel with Dates - Subsc.
 2 x 1Kg Grain Free Chicken - Subsc.
@@ -14567,132 +14922,156 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="11" t="n">
+    <row r="23">
+      <c r="A23" s="11" t="n">
         <v>26891</v>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>Taskeen Moolla</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D20" s="11" t="n">
+      <c r="D23" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E20" s="14" t="n">
+      <c r="E23" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="14" t="n">
         <v>389.2</v>
       </c>
-      <c r="F20" s="14" t="n">
-        <v>25</v>
-      </c>
-      <c r="G20" s="14" t="n">
+      <c r="H23" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="I23" s="14" t="n">
         <v>414.2</v>
       </c>
-      <c r="H20" s="12" t="inlineStr">
+      <c r="J23" s="12" t="inlineStr">
         <is>
           <t>35 x 80g Duck with Tuna Pâté - Subsc.
 23 x Beef Pâté 80g</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="11" t="n">
+    <row r="24">
+      <c r="A24" s="11" t="n">
         <v>41550</v>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>Zak</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D21" s="11" t="n">
+      <c r="D24" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E21" s="14" t="n">
+      <c r="E24" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="14" t="n">
         <v>364</v>
       </c>
-      <c r="F21" s="14" t="n">
+      <c r="H24" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="G21" s="14" t="n">
+      <c r="I24" s="14" t="n">
         <v>414</v>
       </c>
-      <c r="H21" s="12" t="inlineStr">
+      <c r="J24" s="12" t="inlineStr">
         <is>
           <t>4 x Chicken with Banana 1kg
 4 x Turkey with Honey 1kg</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="11" t="n">
+    <row r="25">
+      <c r="A25" s="11" t="n">
         <v>27253</v>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Diana Stepan</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D22" s="11" t="n">
+      <c r="D25" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E22" s="14" t="n">
+      <c r="E25" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="14" t="n">
         <v>275.48</v>
       </c>
-      <c r="F22" s="14" t="n">
+      <c r="H25" s="14" t="n">
         <v>75</v>
       </c>
-      <c r="G22" s="14" t="n">
+      <c r="I25" s="14" t="n">
         <v>350.48</v>
       </c>
-      <c r="H22" s="12" t="inlineStr">
+      <c r="J25" s="12" t="inlineStr">
         <is>
           <t>3 x 1Kg Camel with Quinoa - Subsc.
 2 x Camel with Quinoa 1kg</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="11" t="n">
+    <row r="26">
+      <c r="A26" s="11" t="n">
         <v>40937</v>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>Erika Belaja</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D23" s="11" t="n">
+      <c r="D26" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E23" s="14" t="n">
+      <c r="E26" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="14" t="n">
         <v>133.6</v>
       </c>
-      <c r="F23" s="14" t="n">
+      <c r="H26" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="G23" s="14" t="n">
+      <c r="I26" s="14" t="n">
         <v>183.6</v>
       </c>
-      <c r="H23" s="12" t="inlineStr">
+      <c r="J26" s="12" t="inlineStr">
         <is>
           <t>1 x 1Kg Chicken with Banana - Subsc.
 1 x 1Kg Camel with Dates - Subsc.
@@ -14700,65 +15079,77 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="11" t="n">
+    <row r="27">
+      <c r="A27" s="11" t="n">
         <v>29813</v>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Second Chance Animal Sanctuary</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D24" s="11" t="n">
+      <c r="D27" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="E24" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="14" t="n">
+      <c r="E27" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="14" t="n">
         <v>175</v>
       </c>
-      <c r="G24" s="14" t="n">
+      <c r="I27" s="14" t="n">
         <v>175</v>
       </c>
-      <c r="H24" s="12" t="inlineStr">
+      <c r="J27" s="12" t="inlineStr">
         <is>
           <t>10 x Samples</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="11" t="n">
+    <row r="28">
+      <c r="A28" s="11" t="n">
         <v>42050</v>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>Alessandra Fuscaldo</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D25" s="11" t="n">
+      <c r="D28" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E25" s="14" t="n">
+      <c r="E28" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="14" t="n">
         <v>106.12</v>
       </c>
-      <c r="F25" s="14" t="n">
-        <v>25</v>
-      </c>
-      <c r="G25" s="14" t="n">
+      <c r="H28" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="I28" s="14" t="n">
         <v>131.12</v>
       </c>
-      <c r="H25" s="12" t="inlineStr">
+      <c r="J28" s="12" t="inlineStr">
         <is>
           <t>12 x 80g Duck with Tuna Pâté - Subsc.
 4 x 80g Chicken Pâté - Subsc.
@@ -14766,33 +15157,39 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="11" t="n">
+    <row r="29">
+      <c r="A29" s="11" t="n">
         <v>40709</v>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>Dr. Susan Aylott</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D26" s="11" t="n">
+      <c r="D29" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E26" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="14" t="n">
-        <v>25</v>
-      </c>
-      <c r="G26" s="14" t="n">
-        <v>25</v>
-      </c>
-      <c r="H26" s="12" t="inlineStr">
+      <c r="E29" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="I29" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="J29" s="12" t="inlineStr">
         <is>
           <t>5 x 80g Duck with Tuna Pâté - Subsc.
 5 x 80g Chicken Pâté - Subsc.
@@ -14801,27 +15198,29 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B27" s="13" t="n"/>
-      <c r="C27" s="13" t="n"/>
-      <c r="D27" s="9" t="n">
-        <v>96</v>
-      </c>
-      <c r="E27" s="10" t="n">
-        <v>27641.35</v>
-      </c>
-      <c r="F27" s="10" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G27" s="10" t="n">
-        <v>29741.35</v>
-      </c>
-      <c r="H27" s="13" t="n"/>
+      <c r="B30" s="13" t="n"/>
+      <c r="C30" s="13" t="n"/>
+      <c r="D30" s="9" t="n">
+        <v>125</v>
+      </c>
+      <c r="E30" s="13" t="n"/>
+      <c r="F30" s="13" t="n"/>
+      <c r="G30" s="10" t="n">
+        <v>45693.38</v>
+      </c>
+      <c r="H30" s="10" t="n">
+        <v>2225</v>
+      </c>
+      <c r="I30" s="10" t="n">
+        <v>47918.38</v>
+      </c>
+      <c r="J30" s="13" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>